<commit_message>
fixed test cases in lscbranch
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F8791D-FE8F-43D2-AF51-C28E3B4AD6D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED29ACF-D395-4B1E-998E-1649FB106438}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="6" activeTab="11" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="13" activeTab="17" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -1875,8 +1875,8 @@
       <c r="B8" t="s">
         <v>77</v>
       </c>
-      <c r="C8" t="s">
-        <v>78</v>
+      <c r="C8" s="11" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1896,6 +1896,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1" tooltip="Basic Field Grant Office" display="https://test7-internal--lsc--c.cs92.visual.force.com/0013F00000UJsYpQAL" xr:uid="{9CBF36DE-4B3A-4BB6-A4BE-813F9EE8E219}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
made changes in sanity and excel sheet
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Product\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419FEF93-22FC-46CE-8724-DD2C01B6FDFF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD325C96-417C-4F36-8C61-AD4014A1C685}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="20" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="137">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -465,6 +465,21 @@
   </si>
   <si>
     <t>fieldExternalOrganization__c</t>
+  </si>
+  <si>
+    <t>fieldSubmissionTitle__c</t>
+  </si>
+  <si>
+    <t>fieldScheduleBase__c</t>
+  </si>
+  <si>
+    <t>fieldCalReportingStartDate__c</t>
+  </si>
+  <si>
+    <t>fieldCalReportingEndDate__c</t>
+  </si>
+  <si>
+    <t>fieldFrequency__c</t>
   </si>
 </sst>
 </file>
@@ -922,7 +937,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
         <v>118</v>
@@ -933,7 +948,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>136</v>
       </c>
       <c r="C3" t="s">
         <v>96</v>
@@ -944,7 +959,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>133</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -2657,7 +2672,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
         <v>121</v>
@@ -2668,7 +2683,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>133</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -2679,7 +2694,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>134</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -2690,7 +2705,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>135</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -2701,7 +2716,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>136</v>
       </c>
       <c r="C6" t="s">
         <v>96</v>

</xml_diff>

<commit_message>
Merged PR 15265: Merge prod_lwc_saranjit to LWC_Product_Test
Added Progress Report Changes
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New LWC\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New Project\ProdLWC_Mine\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9735B509-B010-45FE-9C20-A57B279E076C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E3DC1B-8747-439E-BD22-3C6563219FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="35" activeTab="36" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="53" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -45,8 +45,8 @@
     <sheet name="Grant_Edition1" sheetId="30" r:id="rId30"/>
     <sheet name="Grant_Edition_Comp_Focus_No" sheetId="60" r:id="rId31"/>
     <sheet name="Edition" sheetId="1" r:id="rId32"/>
-    <sheet name="Edition_ByAppFocusYes" sheetId="66" r:id="rId33"/>
-    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId34"/>
+    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId33"/>
+    <sheet name="Edition_ByAppFocusYes" sheetId="66" r:id="rId34"/>
     <sheet name="Grant_Creation4" sheetId="36" r:id="rId35"/>
     <sheet name="Grant_Creation3" sheetId="35" r:id="rId36"/>
     <sheet name="Grant_Creation1" sheetId="31" r:id="rId37"/>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1658" uniqueCount="160">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -372,6 +372,9 @@
     <t>Monthly</t>
   </si>
   <si>
+    <t>fieldInternalOrganization__c</t>
+  </si>
+  <si>
     <t>Automation Permanent Internal Program</t>
   </si>
   <si>
@@ -435,6 +438,21 @@
     <t xml:space="preserve">Automation Runtime Payment Request </t>
   </si>
   <si>
+    <t>fieldProjectTitle__c</t>
+  </si>
+  <si>
+    <t>fieldProjectPeriodStartDate__c</t>
+  </si>
+  <si>
+    <t>fieldProjectPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>fieldProgram__c</t>
+  </si>
+  <si>
+    <t>fieldExternalOrganization__c</t>
+  </si>
+  <si>
     <t>Automation SPI3</t>
   </si>
   <si>
@@ -453,7 +471,46 @@
     <t>Department of Health</t>
   </si>
   <si>
+    <t>fieldIsMatchRequired__c</t>
+  </si>
+  <si>
+    <t>fieldGranteeMatch__c</t>
+  </si>
+  <si>
+    <t>fieldLaverageAllowed__c</t>
+  </si>
+  <si>
+    <t>fieldIsProgramIncomeAnticipated__c</t>
+  </si>
+  <si>
+    <t>fieldIsAdvancePermitted__c</t>
+  </si>
+  <si>
+    <t>fieldIsBuildUpFunctionality__c</t>
+  </si>
+  <si>
+    <t>fieldIsGoalsRequired__c</t>
+  </si>
+  <si>
+    <t>fieldKPIsRequired__c</t>
+  </si>
+  <si>
+    <t>fieldAreExpensesBuildIUpLevel__c</t>
+  </si>
+  <si>
+    <t>fieldRiskAssessmentRequired__c</t>
+  </si>
+  <si>
+    <t>fieldFocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>fieldGrantType__c</t>
+  </si>
+  <si>
     <t>Directed</t>
+  </si>
+  <si>
+    <t>fieldAllocationLevel__c</t>
   </si>
   <si>
     <t>N/A</t>
@@ -526,7 +583,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -571,6 +628,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="5"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color rgb="FF202124"/>
       <name val="Consolas"/>
@@ -604,22 +667,9 @@
       <family val="3"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF222222"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF202124"/>
-      <name val="Consolas"/>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
       <family val="3"/>
     </font>
   </fonts>
@@ -663,9 +713,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -694,21 +744,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1025,10 +1071,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.81640625" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1050,7 +1096,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1084,10 +1130,10 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB5817C-6282-474A-8544-903751FEE950}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1106,10 +1152,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1127,8 +1173,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1138,8 +1184,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1161,10 +1207,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1175,14 +1221,14 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>71</v>
       </c>
       <c r="C9" t="s">
@@ -1197,10 +1243,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED68E7CE-CC8D-4336-AB4D-FCC4D911F847}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36.54296875" customWidth="1"/>
-    <col min="3" max="3" width="39.1796875" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1219,10 +1265,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1240,8 +1286,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1251,8 +1297,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1274,10 +1320,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1285,21 +1331,21 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>71</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1310,10 +1356,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E64C7070-1AFC-4706-8E5B-A6B0F56D48B4}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1332,10 +1378,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1353,8 +1399,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1364,8 +1410,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1387,7 +1433,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -1398,17 +1444,17 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>71</v>
       </c>
       <c r="C9" t="s">
@@ -1423,11 +1469,11 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1446,10 +1492,10 @@
         <v>8</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1467,8 +1513,8 @@
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4" s="9">
         <v>0</v>
@@ -1478,8 +1524,8 @@
       <c r="A5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5" s="9">
         <v>3650</v>
@@ -1501,7 +1547,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>69</v>
@@ -1515,7 +1561,7 @@
         <v>70</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1526,7 +1572,7 @@
         <v>71</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1538,10 +1584,10 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1564,7 +1610,7 @@
         <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1582,8 +1628,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1593,8 +1639,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1616,7 +1662,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -1630,7 +1676,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1652,9 +1698,9 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="35.81640625" style="21" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1662,7 +1708,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -1673,18 +1719,18 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="13" t="s">
         <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" t="s">
         <v>66</v>
       </c>
       <c r="C3" t="s">
@@ -1695,8 +1741,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="22" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1706,8 +1752,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>365</v>
@@ -1717,7 +1763,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" t="s">
         <v>67</v>
       </c>
       <c r="C6" t="s">
@@ -1728,8 +1774,8 @@
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="20" t="s">
-        <v>99</v>
+      <c r="B7" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -1739,18 +1785,18 @@
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" t="s">
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" t="s">
         <v>71</v>
       </c>
       <c r="C9" t="s">
@@ -1766,7 +1812,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -1791,7 +1837,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1820,8 +1866,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
-        <v>136</v>
+      <c r="B5" s="20" t="s">
+        <v>155</v>
       </c>
       <c r="C5">
         <v>-300</v>
@@ -1831,8 +1877,8 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>137</v>
+      <c r="B6" s="20" t="s">
+        <v>156</v>
       </c>
       <c r="C6">
         <v>1000</v>
@@ -1846,10 +1892,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
-    <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1912,7 +1958,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -1989,22 +2035,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>121</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2016,10 +2062,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2160,7 +2206,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C13">
         <v>15</v>
@@ -2170,22 +2216,22 @@
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>121</v>
+      <c r="B14" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>119</v>
+      <c r="B15" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2196,10 +2242,10 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2339,22 +2385,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>121</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2365,9 +2411,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2507,22 +2553,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>121</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2533,10 +2579,10 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E65B36E-C406-494A-B0E2-B964D6868C97}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2680,9 +2726,9 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0640EED7-D2C9-455A-A602-2DFF3D455D0D}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2701,8 +2747,8 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>74</v>
+      <c r="B2" s="14" t="s">
+        <v>124</v>
       </c>
       <c r="C2" t="s">
         <v>37</v>
@@ -2712,8 +2758,8 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>75</v>
+      <c r="B3" s="14" t="s">
+        <v>125</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -2723,8 +2769,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>76</v>
+      <c r="B4" s="14" t="s">
+        <v>126</v>
       </c>
       <c r="C4" t="s">
         <v>37</v>
@@ -2734,8 +2780,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>77</v>
+      <c r="B5" s="14" t="s">
+        <v>127</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
@@ -2745,8 +2791,8 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>78</v>
+      <c r="B6" s="14" t="s">
+        <v>128</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -2756,8 +2802,8 @@
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>79</v>
+      <c r="B7" s="14" t="s">
+        <v>129</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
@@ -2767,8 +2813,8 @@
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>80</v>
+      <c r="B8" s="14" t="s">
+        <v>130</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -2778,8 +2824,8 @@
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>81</v>
+      <c r="B9" s="14" t="s">
+        <v>131</v>
       </c>
       <c r="C9" t="s">
         <v>37</v>
@@ -2789,8 +2835,8 @@
       <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>82</v>
+      <c r="B10" s="14" t="s">
+        <v>132</v>
       </c>
       <c r="C10" t="s">
         <v>37</v>
@@ -2800,8 +2846,8 @@
       <c r="A11" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>83</v>
+      <c r="B11" s="14" t="s">
+        <v>133</v>
       </c>
       <c r="C11" t="s">
         <v>30</v>
@@ -2811,8 +2857,8 @@
       <c r="A12" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="13" t="s">
-        <v>86</v>
+      <c r="B12" s="14" t="s">
+        <v>134</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
@@ -2822,22 +2868,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>118</v>
+      <c r="B13" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>119</v>
+      <c r="B14" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2848,10 +2894,10 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8BBCA7-84E5-468D-9593-DDDDFFC181D9}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2913,7 +2959,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -2990,22 +3036,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>122</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>123</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3016,10 +3062,10 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD6EACD2-E384-4732-A671-45DCB7110B6D}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3081,7 +3127,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -3158,22 +3204,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>122</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>123</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3184,10 +3230,10 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20FA9E41-6948-44F3-A81E-083ABEFAA1FF}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3249,7 +3295,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -3326,22 +3372,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>122</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>124</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3352,10 +3398,10 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77BC984D-E65A-4F8B-8C91-6B719CF3E96D}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="25.81640625" customWidth="1"/>
-    <col min="3" max="3" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3417,7 +3463,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -3494,22 +3540,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>122</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>124</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3520,10 +3566,10 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A20FB1D9-E5BB-4D84-B22C-428D1F9F758E}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3585,7 +3631,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -3662,22 +3708,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>118</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -3688,10 +3734,10 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AD4597-E451-4F1E-8711-FD7052A2DCDF}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3753,7 +3799,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -3830,22 +3876,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>118</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -3856,9 +3902,9 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{234E1846-B96C-4D8F-A545-8F81DE4A8384}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3921,7 +3967,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -3998,22 +4044,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>118</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -4024,9 +4070,9 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB025003-6BB5-454C-A664-0A8352B6971A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4089,7 +4135,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -4166,22 +4212,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>121</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -4191,10 +4237,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28.26953125" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4214,10 +4260,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -4235,8 +4281,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>-3650</v>
@@ -4246,8 +4292,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>900</v>
@@ -4269,7 +4315,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -4283,7 +4329,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -4294,6 +4340,17 @@
         <v>71</v>
       </c>
       <c r="C9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4305,10 +4362,10 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
-    <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4371,7 +4428,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -4448,22 +4505,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>121</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -4474,9 +4531,9 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19D4AB1B-6626-42AC-8E84-B372170101F0}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4539,7 +4596,7 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>78</v>
       </c>
       <c r="C6" t="s">
@@ -4616,22 +4673,22 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>121</v>
+      <c r="B13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>119</v>
+      <c r="B14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -4642,10 +4699,10 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.81640625" customWidth="1"/>
-    <col min="2" max="2" width="32.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4676,10 +4733,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4687,7 +4744,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="C4">
         <v>1234</v>
@@ -4698,7 +4755,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C5">
         <v>123</v>
@@ -4708,8 +4765,8 @@
       <c r="A6" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>133</v>
+      <c r="B6" s="14" t="s">
+        <v>152</v>
       </c>
       <c r="C6">
         <v>150</v>
@@ -4722,12 +4779,12 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E1CF92D-A01C-46CA-ABC1-C62A79070058}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.453125" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="1" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4757,10 +4814,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4768,7 +4825,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="C4">
         <v>1234</v>
@@ -4779,7 +4836,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C5">
         <v>123</v>
@@ -4790,7 +4847,7 @@
         <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="C6">
         <v>3650</v>
@@ -4801,9 +4858,20 @@
         <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="C7">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C8">
         <v>2000</v>
       </c>
     </row>
@@ -4813,12 +4881,13 @@
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{757E1FCF-2686-4EA9-B6EB-44427A757385}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="28.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4848,10 +4917,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4859,7 +4928,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="C4">
         <v>1234</v>
@@ -4870,7 +4939,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C5">
         <v>123</v>
@@ -4881,7 +4950,7 @@
         <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="C6">
         <v>3650</v>
@@ -4892,20 +4961,9 @@
         <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="C7">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B8" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8">
         <v>2000</v>
       </c>
     </row>
@@ -4917,11 +4975,11 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4950,8 +5008,8 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>126</v>
+      <c r="B3" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -4961,8 +5019,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>127</v>
+      <c r="B4" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -4984,7 +5042,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
         <v>69</v>
@@ -4998,7 +5056,7 @@
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5020,7 +5078,7 @@
         <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -5032,10 +5090,10 @@
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="38.81640625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5064,8 +5122,8 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>126</v>
+      <c r="B3" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -5075,8 +5133,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>127</v>
+      <c r="B4" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -5098,7 +5156,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
         <v>69</v>
@@ -5112,7 +5170,7 @@
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5134,7 +5192,7 @@
         <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -5142,7 +5200,7 @@
     </row>
     <row r="19" spans="7:7">
       <c r="G19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -5154,10 +5212,10 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5187,7 +5245,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -5198,7 +5256,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -5220,7 +5278,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
         <v>69</v>
@@ -5234,7 +5292,7 @@
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5256,12 +5314,12 @@
         <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="7:7">
       <c r="G19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -5272,10 +5330,10 @@
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5298,7 +5356,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5317,7 +5375,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -5328,10 +5386,10 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C5">
-        <v>3650</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5343,6 +5401,17 @@
       </c>
       <c r="C6" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -5353,11 +5422,11 @@
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.81640625" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5379,7 +5448,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5398,7 +5467,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -5409,10 +5478,10 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C5">
-        <v>3650</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5424,6 +5493,17 @@
       </c>
       <c r="C6" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -5435,9 +5515,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5460,7 +5540,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5498,7 +5578,7 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -5523,7 +5603,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5564,10 +5644,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5575,7 +5655,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -5589,11 +5669,11 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5825,11 +5905,11 @@
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.1796875" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5863,11 +5943,11 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5934,10 +6014,10 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5959,7 +6039,7 @@
         <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5970,7 +6050,7 @@
         <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5992,11 +6072,11 @@
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6018,7 +6098,7 @@
         <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6029,7 +6109,7 @@
         <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6051,10 +6131,10 @@
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6073,10 +6153,10 @@
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6084,7 +6164,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -6099,10 +6179,10 @@
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F460C7BE-6B78-4C1D-8F43-EB5ECFF94C59}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6121,10 +6201,10 @@
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6132,7 +6212,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -6146,11 +6226,11 @@
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6348,15 +6428,15 @@
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
-    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1796875" customWidth="1"/>
-    <col min="7" max="7" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -6547,11 +6627,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="31.81640625" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6573,7 +6653,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6606,11 +6686,11 @@
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B06FA50-0033-457A-9572-B9C40BB74376}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="40.1796875" customWidth="1"/>
+    <col min="3" max="3" width="40.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6640,7 +6720,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -6651,7 +6731,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -6672,11 +6752,11 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>99</v>
+      <c r="B6" s="14" t="s">
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -6687,7 +6767,7 @@
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -6705,11 +6785,11 @@
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -6720,10 +6800,10 @@
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6877,10 +6957,10 @@
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.81640625" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6902,18 +6982,18 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6943,7 +7023,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -6954,7 +7034,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -6969,11 +7049,11 @@
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" customWidth="1"/>
-    <col min="2" max="2" width="32.81640625" customWidth="1"/>
-    <col min="3" max="3" width="49.81640625" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.85546875" customWidth="1"/>
+    <col min="3" max="3" width="49.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6995,18 +7075,18 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7036,7 +7116,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7047,7 +7127,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>3700</v>
@@ -7061,11 +7141,11 @@
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="28.1796875" customWidth="1"/>
-    <col min="3" max="3" width="29.1796875" customWidth="1"/>
+    <col min="1" max="1" width="24.85546875" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7087,18 +7167,18 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7128,7 +7208,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7139,7 +7219,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>365</v>
@@ -7153,11 +7233,11 @@
 <file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.81640625" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="29.1796875" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7179,18 +7259,18 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7220,7 +7300,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7231,7 +7311,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>365</v>
@@ -7245,7 +7325,7 @@
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -7270,7 +7350,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7281,7 +7361,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7311,7 +7391,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7322,7 +7402,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>365</v>
@@ -7337,10 +7417,10 @@
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7362,18 +7442,18 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7403,7 +7483,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7414,7 +7494,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>365</v>
@@ -7428,9 +7508,9 @@
 <file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7453,7 +7533,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7483,7 +7563,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -7494,7 +7574,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C6">
         <v>365</v>
@@ -7508,7 +7588,7 @@
 <file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -7533,7 +7613,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7563,7 +7643,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C5">
         <v>-25</v>
@@ -7574,7 +7654,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C6">
         <v>365</v>
@@ -7588,7 +7668,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
@@ -7610,10 +7690,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7631,8 +7711,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -7642,8 +7722,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -7665,7 +7745,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -7679,7 +7759,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -7687,7 +7767,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
         <v>72</v>
@@ -7702,7 +7782,7 @@
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -7727,14 +7807,14 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -7768,7 +7848,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7779,7 +7859,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>480</v>
@@ -7793,7 +7873,7 @@
 <file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2A00-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
@@ -7818,18 +7898,18 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7859,7 +7939,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -7870,7 +7950,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C7">
         <v>460</v>
@@ -7878,16 +7958,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{129E2C7B-C704-47A8-8150-6E03A592DEEB}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" customWidth="1"/>
-    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7907,10 +7988,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7928,8 +8009,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -7939,8 +8020,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -7962,7 +8043,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -7976,7 +8057,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -7998,9 +8079,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="25.453125" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8020,10 +8101,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -8041,8 +8122,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -8052,8 +8133,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -8075,7 +8156,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -8089,7 +8170,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -8111,10 +8192,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DED3A87-6AC6-43AA-AE6F-BF4F74835A6A}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8133,10 +8214,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -8154,8 +8235,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>114</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -8165,14 +8246,14 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>115</v>
       </c>
       <c r="C5">
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1">
+    <row r="6" spans="1:3" ht="15.75" thickBot="1">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -8183,15 +8264,15 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1">
+    <row r="7" spans="1:3" ht="15.75" thickBot="1">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>116</v>
+        <v>91</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -8199,21 +8280,21 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>120</v>
+        <v>116</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="14" t="s">
+      <c r="B9" s="14" t="s">
         <v>117</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -8228,9 +8309,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="29.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8253,7 +8334,7 @@
         <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -8271,8 +8352,8 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>126</v>
+      <c r="B4" s="14" t="s">
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -8282,8 +8363,8 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>127</v>
+      <c r="B5" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -8305,7 +8386,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>69</v>
@@ -8319,7 +8400,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:3">

</xml_diff>

<commit_message>
script updation for organization risk assessment module
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cleanup_Projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santosh J\REI Projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B35B3F2-F0EF-40A3-8F1A-C57011AEC15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65851922-517F-44C9-85FA-6285CC873BC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="46" activeTab="46" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -109,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2051" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2051" uniqueCount="163">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -595,6 +595,9 @@
   </si>
   <si>
     <t>Automation Runtime Financial Report</t>
+  </si>
+  <si>
+    <t>Automation Permanent Organization for Risk Assessment</t>
   </si>
 </sst>
 </file>
@@ -1099,10 +1102,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.88671875" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1158,10 +1161,10 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F0C9D9D-E322-4515-BDD4-A1A8F3618247}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1359,10 +1362,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF74A305-566F-4C32-B26D-8047485FB6C5}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1538,10 +1541,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89D5F24D-5E2D-4584-B902-FBD053FD9969}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1739,10 +1742,10 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CF4B69D-1D60-40C4-BB2E-53842135881E}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1940,10 +1943,10 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DFE1A96-148E-4EFE-B3D1-6648137C24F7}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2053,10 +2056,10 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B648CAAD-4299-4CA9-A9AD-89C2F01011CD}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2166,10 +2169,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB5817C-6282-474A-8544-903751FEE950}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2279,10 +2282,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED68E7CE-CC8D-4336-AB4D-FCC4D911F847}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="36.5546875" customWidth="1"/>
-    <col min="3" max="3" width="39.109375" customWidth="1"/>
+    <col min="2" max="2" width="36.54296875" customWidth="1"/>
+    <col min="3" max="3" width="39.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2392,10 +2395,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E64C7070-1AFC-4706-8E5B-A6B0F56D48B4}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2505,11 +2508,11 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2620,9 +2623,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2788,10 +2791,10 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2902,9 +2905,9 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3016,7 +3019,7 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -3096,10 +3099,10 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3266,10 +3269,10 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3446,10 +3449,10 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3615,10 +3618,10 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E65B36E-C406-494A-B0E2-B964D6868C97}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3762,9 +3765,9 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0640EED7-D2C9-455A-A602-2DFF3D455D0D}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3930,10 +3933,10 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8BBCA7-84E5-468D-9593-DDDDFFC181D9}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4098,10 +4101,10 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD6EACD2-E384-4732-A671-45DCB7110B6D}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4266,9 +4269,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4379,10 +4382,10 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20FA9E41-6948-44F3-A81E-083ABEFAA1FF}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4547,10 +4550,10 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77BC984D-E65A-4F8B-8C91-6B719CF3E96D}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="25.88671875" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" customWidth="1"/>
+    <col min="2" max="2" width="25.90625" customWidth="1"/>
+    <col min="3" max="3" width="35.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4715,10 +4718,10 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A20FB1D9-E5BB-4D84-B22C-428D1F9F758E}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4883,10 +4886,10 @@
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AD4597-E451-4F1E-8711-FD7052A2DCDF}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5051,9 +5054,9 @@
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{234E1846-B96C-4D8F-A545-8F81DE4A8384}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5219,9 +5222,9 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB025003-6BB5-454C-A664-0A8352B6971A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5387,10 +5390,10 @@
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5556,10 +5559,10 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4921DA-1B28-4302-A76B-C303820C11A2}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5713,9 +5716,9 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19D4AB1B-6626-42AC-8E84-B372170101F0}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5881,10 +5884,10 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.90625" customWidth="1"/>
+    <col min="2" max="2" width="32.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5963,9 +5966,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6026,9 +6029,9 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="28.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6128,7 +6131,7 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{217EED23-ED46-4B3B-8704-FA540DCAAEE6}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
@@ -6156,7 +6159,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.2" customHeight="1">
+    <row r="3" spans="1:3" ht="16.25" customHeight="1">
       <c r="A3" s="22" t="s">
         <v>8</v>
       </c>
@@ -6200,7 +6203,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="12.6" customHeight="1">
+    <row r="7" spans="1:3" ht="12.65" customHeight="1">
       <c r="A7" s="22" t="s">
         <v>8</v>
       </c>
@@ -6211,7 +6214,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.6" customHeight="1">
+    <row r="8" spans="1:3" ht="15.65" customHeight="1">
       <c r="A8" s="22" t="s">
         <v>8</v>
       </c>
@@ -6255,7 +6258,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.2" customHeight="1">
+    <row r="12" spans="1:3" ht="16.25" customHeight="1">
       <c r="A12" s="22" t="s">
         <v>8</v>
       </c>
@@ -6288,7 +6291,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.6" customHeight="1">
+    <row r="15" spans="1:3" ht="12.65" customHeight="1">
       <c r="A15" s="22" t="s">
         <v>8</v>
       </c>
@@ -6329,10 +6332,10 @@
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73A04F39-DE0D-44C3-97CE-7095515ADE47}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6442,10 +6445,10 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8F35E33-E3A9-4945-BE52-304F10C18E9D}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6544,10 +6547,10 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5311052-4A83-4BE6-A651-A8D0B3D0FF12}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6646,10 +6649,10 @@
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C802F615-EB92-4BFC-87EF-94C5A3A77613}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6759,11 +6762,11 @@
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{757E1FCF-2686-4EA9-B6EB-44427A757385}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6851,11 +6854,11 @@
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6921,7 +6924,7 @@
         <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -6966,10 +6969,10 @@
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="3" max="3" width="38.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7088,10 +7091,10 @@
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7207,11 +7210,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="31.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7266,9 +7269,9 @@
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7358,10 +7361,10 @@
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.88671875" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7450,7 +7453,7 @@
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -7541,11 +7544,11 @@
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7777,11 +7780,11 @@
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" customWidth="1"/>
+    <col min="3" max="3" width="20.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7815,11 +7818,11 @@
 <file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7886,10 +7889,10 @@
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.109375" customWidth="1"/>
+    <col min="2" max="2" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7944,11 +7947,11 @@
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8003,10 +8006,10 @@
 <file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8051,10 +8054,10 @@
 <file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F460C7BE-6B78-4C1D-8F43-EB5ECFF94C59}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8098,7 +8101,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
@@ -8212,11 +8215,11 @@
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8414,15 +8417,15 @@
 <file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.109375" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.08984375" customWidth="1"/>
+    <col min="2" max="2" width="9.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" customWidth="1"/>
+    <col min="6" max="6" width="12.08984375" customWidth="1"/>
+    <col min="7" max="7" width="13.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -8613,11 +8616,11 @@
 <file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B06FA50-0033-457A-9572-B9C40BB74376}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" customWidth="1"/>
+    <col min="3" max="3" width="40.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8727,10 +8730,10 @@
 <file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8884,10 +8887,10 @@
 <file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.88671875" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8976,11 +8979,11 @@
 <file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" customWidth="1"/>
-    <col min="3" max="3" width="49.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.90625" customWidth="1"/>
+    <col min="2" max="2" width="32.90625" customWidth="1"/>
+    <col min="3" max="3" width="49.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9068,11 +9071,11 @@
 <file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.88671875" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="24.90625" customWidth="1"/>
+    <col min="2" max="2" width="28.08984375" customWidth="1"/>
+    <col min="3" max="3" width="29.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9160,11 +9163,11 @@
 <file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="1" max="1" width="27.90625" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="29.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9252,7 +9255,7 @@
 <file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -9344,10 +9347,10 @@
 <file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9435,9 +9438,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9548,9 +9551,9 @@
 <file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9628,7 +9631,7 @@
 <file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -9708,7 +9711,7 @@
 <file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -9799,7 +9802,7 @@
 <file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2A00-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
@@ -9891,10 +9894,10 @@
 <file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{129E2C7B-C704-47A8-8150-6E03A592DEEB}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" customWidth="1"/>
+    <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10005,10 +10008,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DED3A87-6AC6-43AA-AE6F-BF4F74835A6A}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -10122,9 +10125,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
commit testing for FFATA
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MergeOrg2_Proj\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16680058-28D8-45E8-B6BC-74AE4C1EFC66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{298335C4-9D98-462C-90B2-50E98C45C0B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -608,13 +608,13 @@
     <t>WASHINGTON CENTER FOR DEAF AND HARD OF HEARING YOUTH</t>
   </si>
   <si>
-    <t>Automation Runtime New FFATA Awards</t>
-  </si>
-  <si>
-    <t>Automation Runtime New FFATA Awards with Two Funding Source</t>
-  </si>
-  <si>
-    <t>Automation Runtime New FFATA Awards with Single Funding Source</t>
+    <t>Academic Intervention for Nonpublic Schools</t>
+  </si>
+  <si>
+    <t>STEM Incentive Program</t>
+  </si>
+  <si>
+    <t>Tuition Assistance Program</t>
   </si>
 </sst>
 </file>

</xml_diff>